<commit_message>
memperbaiki tampilan admin inventory dan menginput buffer stock
</commit_message>
<xml_diff>
--- a/python/Dataset_Forecasting_ARIMA_Lengkap.xlsx
+++ b/python/Dataset_Forecasting_ARIMA_Lengkap.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fauzan\coba coba arima\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\skripsi_forecasting\python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA418874-FEC0-4894-ABE8-4BB91B6735F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D98618A-74B7-4AB8-8BFD-613765813136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="75">
   <si>
     <t>Date</t>
   </si>
@@ -164,6 +164,99 @@
   </si>
   <si>
     <t>jumlah</t>
+  </si>
+  <si>
+    <t>GB-BB-10</t>
+  </si>
+  <si>
+    <t>GB-BB-30</t>
+  </si>
+  <si>
+    <t>GB-CNF-30</t>
+  </si>
+  <si>
+    <t>GB-CNF-10</t>
+  </si>
+  <si>
+    <t>GB-CNF-100</t>
+  </si>
+  <si>
+    <t>GB-CNF-250</t>
+  </si>
+  <si>
+    <t>GB-DS-30</t>
+  </si>
+  <si>
+    <t>GB-DS-10</t>
+  </si>
+  <si>
+    <t>GB-DS-100</t>
+  </si>
+  <si>
+    <t>GB-GF-30</t>
+  </si>
+  <si>
+    <t>GB-GF-10</t>
+  </si>
+  <si>
+    <t>GB-GF-250</t>
+  </si>
+  <si>
+    <t>GB-IB-30</t>
+  </si>
+  <si>
+    <t>GB-IB-10</t>
+  </si>
+  <si>
+    <t>GB-IB-100</t>
+  </si>
+  <si>
+    <t>GB-JOY-30</t>
+  </si>
+  <si>
+    <t>GB-JOY-10</t>
+  </si>
+  <si>
+    <t>GB-JOY-100</t>
+  </si>
+  <si>
+    <t>GB-LDR-30</t>
+  </si>
+  <si>
+    <t>GB-LDR-10</t>
+  </si>
+  <si>
+    <t>GB-LDR-250</t>
+  </si>
+  <si>
+    <t>GB-MYB-30</t>
+  </si>
+  <si>
+    <t>GB-MYB-10</t>
+  </si>
+  <si>
+    <t>GB-MYB-100</t>
+  </si>
+  <si>
+    <t>GB-TC-30</t>
+  </si>
+  <si>
+    <t>GB-TC-10</t>
+  </si>
+  <si>
+    <t>GB-TC-250</t>
+  </si>
+  <si>
+    <t>GB-TP-TV</t>
+  </si>
+  <si>
+    <t>GB-TP-CC</t>
+  </si>
+  <si>
+    <t>GB-DS-250</t>
+  </si>
+  <si>
+    <t>GB-TP-NB</t>
   </si>
 </sst>
 </file>
@@ -547,10 +640,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -559,31 +652,31 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>72</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>15</v>
@@ -592,67 +685,67 @@
         <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>27</v>
+        <v>63</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>33</v>
+        <v>68</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="AM1" s="1" t="s">
         <v>38</v>

</xml_diff>